<commit_message>
Update research sector (VDS_s) 0.xlsx
</commit_message>
<xml_diff>
--- a/clustering/sepsectors/research sector (VDS_s) 0.xlsx
+++ b/clustering/sepsectors/research sector (VDS_s) 0.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="17">
   <si>
     <t>sector</t>
   </si>
@@ -471,7 +471,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G55"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="120.28515625" customWidth="1"/>
@@ -789,7 +789,7 @@
         <v>1093853.40159167</v>
       </c>
     </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B17" s="6" t="s">
         <v>14</v>
       </c>
@@ -810,7 +810,7 @@
         <v>2.5947743971152693E-3</v>
       </c>
     </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B18" s="6" t="s">
         <v>15</v>
       </c>
@@ -831,7 +831,7 @@
         <v>2.2454820234090326E-3</v>
       </c>
     </row>
-    <row r="20" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B20" s="6" t="s">
         <v>16</v>
       </c>
@@ -850,6 +850,540 @@
       <c r="G20" s="3">
         <f t="shared" si="2"/>
         <v>1.1555534045986038</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G24" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C25" s="2">
+        <v>2024</v>
+      </c>
+      <c r="D25" s="3">
+        <v>2312764.5271400302</v>
+      </c>
+      <c r="E25" s="3">
+        <v>35420.059524999997</v>
+      </c>
+      <c r="F25" s="4">
+        <v>5.6205038026400662E-3</v>
+      </c>
+      <c r="G25" s="4">
+        <v>1.8864917830766969E-3</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C26" s="2">
+        <v>2023</v>
+      </c>
+      <c r="D26" s="3">
+        <v>2056038.0691327541</v>
+      </c>
+      <c r="E26" s="3">
+        <v>35306.169047820003</v>
+      </c>
+      <c r="F26" s="4">
+        <v>7.4585983781851224E-3</v>
+      </c>
+      <c r="G26" s="4">
+        <v>1.5495337612500891E-3</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C27" s="2">
+        <v>2022</v>
+      </c>
+      <c r="D27" s="3">
+        <v>1713109.9518803279</v>
+      </c>
+      <c r="E27" s="3">
+        <v>77023.192478700003</v>
+      </c>
+      <c r="F27" s="4">
+        <v>9.4864560705148846E-3</v>
+      </c>
+      <c r="G27" s="4">
+        <v>3.0572532777723999E-3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C28" s="2">
+        <v>2021</v>
+      </c>
+      <c r="D28" s="3">
+        <v>1230284.2821290109</v>
+      </c>
+      <c r="E28" s="3">
+        <v>94580.340012330009</v>
+      </c>
+      <c r="F28" s="4">
+        <v>4.1181927359240046E-3</v>
+      </c>
+      <c r="G28" s="4">
+        <v>2.9431664964802489E-3</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B30" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D30" s="3">
+        <f>AVERAGE(D25:D26)</f>
+        <v>2184401.2981363921</v>
+      </c>
+      <c r="E30" s="3">
+        <f t="shared" ref="E30:G30" si="3">AVERAGE(E25:E26)</f>
+        <v>35363.114286409997</v>
+      </c>
+      <c r="F30" s="5">
+        <f t="shared" si="3"/>
+        <v>6.5395510904125943E-3</v>
+      </c>
+      <c r="G30" s="5">
+        <f t="shared" si="3"/>
+        <v>1.718012772163393E-3</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B31" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D31" s="3">
+        <f>AVERAGE(D27:D28)</f>
+        <v>1471697.1170046693</v>
+      </c>
+      <c r="E31" s="3">
+        <f t="shared" ref="E31:G31" si="4">AVERAGE(E27:E28)</f>
+        <v>85801.766245514998</v>
+      </c>
+      <c r="F31" s="5">
+        <f t="shared" si="4"/>
+        <v>6.8023244032194442E-3</v>
+      </c>
+      <c r="G31" s="5">
+        <f t="shared" si="4"/>
+        <v>3.0002098871263244E-3</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C33" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D33" s="3">
+        <f>D30/D31</f>
+        <v>1.4842736816541999</v>
+      </c>
+      <c r="E33" s="3">
+        <f t="shared" ref="E33:G33" si="5">E30/E31</f>
+        <v>0.4121490248256805</v>
+      </c>
+      <c r="F33" s="3">
+        <f t="shared" si="5"/>
+        <v>0.96137007040086431</v>
+      </c>
+      <c r="G33" s="3">
+        <f t="shared" si="5"/>
+        <v>0.57263086143914699</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E35" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G35" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A36" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C36" s="2">
+        <v>2023</v>
+      </c>
+      <c r="D36" s="3">
+        <v>1177149.00870383</v>
+      </c>
+      <c r="E36" s="3">
+        <v>54257.120220599987</v>
+      </c>
+      <c r="F36" s="4">
+        <v>3.1222927114860181E-2</v>
+      </c>
+      <c r="G36" s="4">
+        <v>4.4066793598312361E-3</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A37" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C37" s="2">
+        <v>2024</v>
+      </c>
+      <c r="D37" s="3">
+        <v>1104497.8864203531</v>
+      </c>
+      <c r="E37" s="3">
+        <v>55926.329561999992</v>
+      </c>
+      <c r="F37" s="4">
+        <v>1.456969533637424E-2</v>
+      </c>
+      <c r="G37" s="4">
+        <v>1.725521704280945E-3</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A38" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C38" s="2">
+        <v>2021</v>
+      </c>
+      <c r="D38" s="3">
+        <v>1083208.9167629869</v>
+      </c>
+      <c r="E38" s="3">
+        <v>110639.49239553</v>
+      </c>
+      <c r="F38" s="4">
+        <v>6.9333248439685724E-3</v>
+      </c>
+      <c r="G38" s="4">
+        <v>1.1143475296256969E-3</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A39" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C39" s="2">
+        <v>2022</v>
+      </c>
+      <c r="D39" s="3">
+        <v>1077864.821598877</v>
+      </c>
+      <c r="E39" s="3">
+        <v>73997.227386940009</v>
+      </c>
+      <c r="F39" s="4">
+        <v>9.7692142174449353E-3</v>
+      </c>
+      <c r="G39" s="4">
+        <v>9.558347653642385E-3</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B41" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D41" s="3">
+        <f>AVERAGE(D36:D37)</f>
+        <v>1140823.4475620915</v>
+      </c>
+      <c r="E41" s="3">
+        <f t="shared" ref="E41:G41" si="6">AVERAGE(E36:E37)</f>
+        <v>55091.724891299993</v>
+      </c>
+      <c r="F41" s="5">
+        <f t="shared" si="6"/>
+        <v>2.2896311225617211E-2</v>
+      </c>
+      <c r="G41" s="5">
+        <f t="shared" si="6"/>
+        <v>3.0661005320560906E-3</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B42" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D42" s="3">
+        <f>AVERAGE(D38:D39)</f>
+        <v>1080536.8691809319</v>
+      </c>
+      <c r="E42" s="3">
+        <f t="shared" ref="E42:G42" si="7">AVERAGE(E38:E39)</f>
+        <v>92318.359891235013</v>
+      </c>
+      <c r="F42" s="5">
+        <f t="shared" si="7"/>
+        <v>8.3512695307067543E-3</v>
+      </c>
+      <c r="G42" s="5">
+        <f t="shared" si="7"/>
+        <v>5.3363475916340412E-3</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C44" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D44" s="3">
+        <f>D41/D42</f>
+        <v>1.0557931710621387</v>
+      </c>
+      <c r="E44" s="3">
+        <f t="shared" ref="E44:G44" si="8">E41/E42</f>
+        <v>0.59675805501967727</v>
+      </c>
+      <c r="F44" s="3">
+        <f t="shared" si="8"/>
+        <v>2.741656360321008</v>
+      </c>
+      <c r="G44" s="3">
+        <f t="shared" si="8"/>
+        <v>0.57456911856021375</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A46" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D46" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E46" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F46" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G46" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A47" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C47" s="2">
+        <v>2024</v>
+      </c>
+      <c r="D47" s="3">
+        <v>729412.67096789309</v>
+      </c>
+      <c r="E47" s="3">
+        <v>60313.34351775</v>
+      </c>
+      <c r="F47" s="4">
+        <v>3.7694938920620688E-4</v>
+      </c>
+      <c r="G47" s="4">
+        <v>1.654533485954597E-3</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A48" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C48" s="2">
+        <v>2021</v>
+      </c>
+      <c r="D48" s="3">
+        <v>648447.24948227091</v>
+      </c>
+      <c r="E48" s="3">
+        <v>22130.276711350001</v>
+      </c>
+      <c r="F48" s="4">
+        <v>1.068848483528837E-2</v>
+      </c>
+      <c r="G48" s="4">
+        <v>8.5913209572516789E-4</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A49" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C49" s="2">
+        <v>2023</v>
+      </c>
+      <c r="D49" s="3">
+        <v>647963.01508706179</v>
+      </c>
+      <c r="E49" s="3">
+        <v>30679.58334573</v>
+      </c>
+      <c r="F49" s="4">
+        <v>6.9744795028248326E-4</v>
+      </c>
+      <c r="G49" s="4">
+        <v>1.104087647419581E-4</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A50" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C50" s="2">
+        <v>2022</v>
+      </c>
+      <c r="D50" s="3">
+        <v>585416.38894337451</v>
+      </c>
+      <c r="E50" s="3">
+        <v>80201.013479729998</v>
+      </c>
+      <c r="F50" s="4">
+        <v>3.0546519921711193E-4</v>
+      </c>
+      <c r="G50" s="4">
+        <v>1.7612261076438901E-4</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B52" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D52" s="3">
+        <f>AVERAGE(D47:D48)</f>
+        <v>688929.960225082</v>
+      </c>
+      <c r="E52" s="3">
+        <f t="shared" ref="E52:G52" si="9">AVERAGE(E47:E48)</f>
+        <v>41221.810114549997</v>
+      </c>
+      <c r="F52" s="5">
+        <f t="shared" si="9"/>
+        <v>5.5327171122472882E-3</v>
+      </c>
+      <c r="G52" s="5">
+        <f t="shared" si="9"/>
+        <v>1.2568327908398826E-3</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B53" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D53" s="3">
+        <f>AVERAGE(D49:D50)</f>
+        <v>616689.70201521809</v>
+      </c>
+      <c r="E53" s="3">
+        <f t="shared" ref="E53:G53" si="10">AVERAGE(E49:E50)</f>
+        <v>55440.298412730001</v>
+      </c>
+      <c r="F53" s="5">
+        <f t="shared" si="10"/>
+        <v>5.0145657474979762E-4</v>
+      </c>
+      <c r="G53" s="5">
+        <f t="shared" si="10"/>
+        <v>1.4326568775317356E-4</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C55" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D55" s="3">
+        <f>D52/D53</f>
+        <v>1.1171419888702492</v>
+      </c>
+      <c r="E55" s="3">
+        <f t="shared" ref="E55:G55" si="11">E52/E53</f>
+        <v>0.74353514130949905</v>
+      </c>
+      <c r="F55" s="3">
+        <f t="shared" si="11"/>
+        <v>11.033292593696363</v>
+      </c>
+      <c r="G55" s="3">
+        <f t="shared" si="11"/>
+        <v>8.7727411256017351</v>
       </c>
     </row>
   </sheetData>
@@ -857,6 +1391,294 @@
     <sortCondition descending="1" ref="D2:D13"/>
   </sortState>
   <conditionalFormatting sqref="D2:D13">
+    <cfRule type="colorScale" priority="32">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E2:E13">
+    <cfRule type="colorScale" priority="31">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F2:F13">
+    <cfRule type="colorScale" priority="30">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G2:G13">
+    <cfRule type="colorScale" priority="29">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D17:D18">
+    <cfRule type="colorScale" priority="28">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E17:E18">
+    <cfRule type="colorScale" priority="27">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F17:F18">
+    <cfRule type="colorScale" priority="26">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G17:G18">
+    <cfRule type="colorScale" priority="25">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D25:D28">
+    <cfRule type="colorScale" priority="24">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E25:E28">
+    <cfRule type="colorScale" priority="23">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F25:F28">
+    <cfRule type="colorScale" priority="22">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G25:G28">
+    <cfRule type="colorScale" priority="21">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D30:D31">
+    <cfRule type="colorScale" priority="20">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E30:E31">
+    <cfRule type="colorScale" priority="19">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F30:F31">
+    <cfRule type="colorScale" priority="18">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G30:G31">
+    <cfRule type="colorScale" priority="17">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D36:D39">
+    <cfRule type="colorScale" priority="16">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E36:E39">
+    <cfRule type="colorScale" priority="15">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F36:F39">
+    <cfRule type="colorScale" priority="14">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G36:G39">
+    <cfRule type="colorScale" priority="13">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D41:D42">
+    <cfRule type="colorScale" priority="12">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E41:E42">
+    <cfRule type="colorScale" priority="11">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F41:F42">
+    <cfRule type="colorScale" priority="10">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G41:G42">
+    <cfRule type="colorScale" priority="9">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D47:D50">
     <cfRule type="colorScale" priority="8">
       <colorScale>
         <cfvo type="min"/>
@@ -868,7 +1690,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E13">
+  <conditionalFormatting sqref="E47:E50">
     <cfRule type="colorScale" priority="7">
       <colorScale>
         <cfvo type="min"/>
@@ -880,7 +1702,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F2:F13">
+  <conditionalFormatting sqref="F47:F50">
     <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="min"/>
@@ -892,7 +1714,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G13">
+  <conditionalFormatting sqref="G47:G50">
     <cfRule type="colorScale" priority="5">
       <colorScale>
         <cfvo type="min"/>
@@ -904,7 +1726,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D17:D18">
+  <conditionalFormatting sqref="D52:D53">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
@@ -916,7 +1738,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E17:E18">
+  <conditionalFormatting sqref="E52:E53">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
@@ -928,7 +1750,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F17:F18">
+  <conditionalFormatting sqref="F52:F53">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -940,7 +1762,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G17:G18">
+  <conditionalFormatting sqref="G52:G53">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>

</xml_diff>